<commit_message>
Mark Publications page as in progress
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/home_content.xlsx
+++ b/data/home_content.xlsx
@@ -1,17 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/63ed0a4e98b474dd/Documents/WESOke_Website/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_EE2CC14B6BBEC26EDE3814D181BE8C3CDAD57EFD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB41E7B8-FD6D-4729-8C8E-75F2047DA0CD}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="3510" yWindow="3645" windowWidth="21600" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sections" sheetId="1" r:id="rId1"/>
     <sheet name="news" sheetId="2" r:id="rId2"/>
     <sheet name="partners" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -27,9 +33,6 @@
     <t>Background</t>
   </si>
   <si>
-    <t>Western Screech-Owls (Megascops kennicottii) were once the most abundant owl across much of coastal British Columbia, Canada. Over the past century their numbers have declined dramatically: a 2006 study (Elliot 2006) estimated an annual rate of decline of 17% on Vancouver Island, and as much as 32% annually in the Lower Mainland. These declines resulted from changing landscapes, habitat loss, and the invasion of Eastern Barred Owls (Strix varia). This project was born out of a need to address the causes of these declines and better understand the ecology of the coastal owls.</t>
-  </si>
-  <si>
     <t>Our Goal</t>
   </si>
   <si>
@@ -70,16 +73,19 @@
   </si>
   <si>
     <t>https://www.pacificmegascops.org/</t>
+  </si>
+  <si>
+    <t>Western Screech-Owls (Megascops kennicottii) were once the most abundant owl across much of coastal British Columbia, Canada. Over the past century their numbers have declined dramatically: a 2006 study (Elliot 2006) estimated an annual rate of decline of 17% on Vancouver Island, and as much as 32% annually in the Lower Mainland. These declines resulted from changing landscapes, habitat loss, and the invasion of Barred Owls (Strix varia) radiating westward from eastern North America. This project was born out of a need to address the causes of these declines and better understand the ecology of the coastal owls. This project is primarily housed through the Quantitative Ecology Lab under the supervision of Dr. Michael Noonan at the University of British Columbia. The project collaborates with many practitioners, governmental bodies, as well as other academics.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd HH:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -128,13 +134,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -172,7 +186,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -206,6 +220,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -240,9 +255,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -415,11 +431,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -427,20 +443,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -449,44 +465,44 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>46182</v>
       </c>
       <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>46220</v>
       </c>
       <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -495,30 +511,30 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>16</v>
-      </c>
-      <c r="C2" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>